<commit_message>
Datos de prueba: el caso imposible replica el ejemplo del cliente
Antes el volumen extra de Distribuidores salía de Mayoristas y lo dejaba
negativo. Ahora la mitad de los SKUs de Soluciones no se vende por
Distribuidores (como el producto grande del ejemplo del cliente) y el
planner le pide a Distribuidores 1.000 kg más de lo que pueden darle sus
SKUs, sacándolos de los otros canales de Soluciones.

Los Excel se generan con fecha fija: regenerar da los mismos bytes. El
test de la base cuenta las celdas leyendo el Excel directo, en vez de
un número fijo que dependía del generador.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/sample/base_mes_anterior.xlsx
+++ b/data/sample/base_mes_anterior.xlsx
@@ -910,20 +910,17 @@
           <t>Azúcar en stick x100</t>
         </is>
       </c>
-      <c r="G22" t="n">
+      <c r="H22" t="n">
         <v>1583</v>
       </c>
-      <c r="H22" t="n">
+      <c r="I22" t="n">
         <v>2208</v>
       </c>
-      <c r="I22" t="n">
+      <c r="J22" t="n">
         <v>3455</v>
       </c>
-      <c r="J22" t="n">
+      <c r="K22" t="n">
         <v>1499</v>
-      </c>
-      <c r="K22" t="n">
-        <v>3998</v>
       </c>
     </row>
     <row r="23">
@@ -936,19 +933,19 @@
         </is>
       </c>
       <c r="G23" t="n">
+        <v>3998</v>
+      </c>
+      <c r="H23" t="n">
         <v>4369</v>
       </c>
-      <c r="H23" t="n">
+      <c r="I23" t="n">
         <v>2293</v>
       </c>
-      <c r="I23" t="n">
+      <c r="J23" t="n">
         <v>1805</v>
       </c>
-      <c r="J23" t="n">
+      <c r="K23" t="n">
         <v>812</v>
-      </c>
-      <c r="K23" t="n">
-        <v>5339</v>
       </c>
     </row>
     <row r="24">
@@ -960,17 +957,17 @@
           <t>Mix capuccino x500</t>
         </is>
       </c>
-      <c r="G24" t="n">
+      <c r="H24" t="n">
+        <v>5339</v>
+      </c>
+      <c r="I24" t="n">
         <v>4515</v>
       </c>
-      <c r="H24" t="n">
+      <c r="J24" t="n">
         <v>5541</v>
       </c>
-      <c r="I24" t="n">
+      <c r="K24" t="n">
         <v>0</v>
-      </c>
-      <c r="K24" t="n">
-        <v>2931</v>
       </c>
     </row>
     <row r="25">
@@ -982,17 +979,14 @@
           <t>Paletina x500</t>
         </is>
       </c>
-      <c r="G25" t="n">
+      <c r="H25" t="n">
+        <v>2931</v>
+      </c>
+      <c r="I25" t="n">
         <v>4738</v>
       </c>
-      <c r="H25" t="n">
+      <c r="J25" t="n">
         <v>1823</v>
-      </c>
-      <c r="J25" t="n">
-        <v>4603</v>
-      </c>
-      <c r="K25" t="n">
-        <v>1806</v>
       </c>
     </row>
     <row r="26">
@@ -1004,17 +998,17 @@
           <t>Azúcar en stick x100</t>
         </is>
       </c>
-      <c r="G26" t="n">
+      <c r="H26" t="n">
+        <v>4603</v>
+      </c>
+      <c r="I26" t="n">
+        <v>1806</v>
+      </c>
+      <c r="J26" t="n">
         <v>4660</v>
       </c>
-      <c r="H26" t="n">
+      <c r="K26" t="n">
         <v>4602</v>
-      </c>
-      <c r="J26" t="n">
-        <v>839</v>
-      </c>
-      <c r="K26" t="n">
-        <v>1453</v>
       </c>
     </row>
     <row r="27">
@@ -1026,14 +1020,11 @@
           <t>Café en grano x500</t>
         </is>
       </c>
+      <c r="H27" t="n">
+        <v>839</v>
+      </c>
       <c r="I27" t="n">
-        <v>1569</v>
-      </c>
-      <c r="J27" t="n">
-        <v>920</v>
-      </c>
-      <c r="K27" t="n">
-        <v>2317</v>
+        <v>1453</v>
       </c>
     </row>
     <row r="28">
@@ -1045,20 +1036,17 @@
           <t>Vaso térmico x100</t>
         </is>
       </c>
-      <c r="G28" t="n">
+      <c r="H28" t="n">
+        <v>1569</v>
+      </c>
+      <c r="I28" t="n">
+        <v>920</v>
+      </c>
+      <c r="J28" t="n">
+        <v>2317</v>
+      </c>
+      <c r="K28" t="n">
         <v>573</v>
-      </c>
-      <c r="H28" t="n">
-        <v>2627</v>
-      </c>
-      <c r="I28" t="n">
-        <v>0</v>
-      </c>
-      <c r="J28" t="n">
-        <v>163</v>
-      </c>
-      <c r="K28" t="n">
-        <v>2155</v>
       </c>
     </row>
     <row r="29">
@@ -1071,13 +1059,19 @@
         </is>
       </c>
       <c r="G29" t="n">
+        <v>2627</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" t="n">
+        <v>163</v>
+      </c>
+      <c r="J29" t="n">
+        <v>2155</v>
+      </c>
+      <c r="K29" t="n">
         <v>176</v>
-      </c>
-      <c r="I29" t="n">
-        <v>2588</v>
-      </c>
-      <c r="K29" t="n">
-        <v>4772</v>
       </c>
     </row>
     <row r="30">
@@ -1089,20 +1083,11 @@
           <t>Café en grano x100</t>
         </is>
       </c>
-      <c r="G30" t="n">
-        <v>2919</v>
-      </c>
-      <c r="H30" t="n">
-        <v>3785</v>
-      </c>
       <c r="I30" t="n">
-        <v>5413</v>
-      </c>
-      <c r="J30" t="n">
-        <v>361</v>
+        <v>2588</v>
       </c>
       <c r="K30" t="n">
-        <v>2639</v>
+        <v>4772</v>
       </c>
     </row>
     <row r="31">
@@ -1115,19 +1100,19 @@
         </is>
       </c>
       <c r="G31" t="n">
-        <v>4916</v>
+        <v>2919</v>
       </c>
       <c r="H31" t="n">
-        <v>5587</v>
+        <v>3785</v>
       </c>
       <c r="I31" t="n">
-        <v>5673</v>
+        <v>5413</v>
       </c>
       <c r="J31" t="n">
-        <v>4156</v>
+        <v>361</v>
       </c>
       <c r="K31" t="n">
-        <v>2110</v>
+        <v>2639</v>
       </c>
     </row>
     <row r="32">
@@ -1139,17 +1124,17 @@
           <t>Tapa para vaso x50</t>
         </is>
       </c>
-      <c r="G32" t="n">
-        <v>2968</v>
+      <c r="H32" t="n">
+        <v>4916</v>
       </c>
       <c r="I32" t="n">
-        <v>243</v>
+        <v>5587</v>
       </c>
       <c r="J32" t="n">
-        <v>2757</v>
+        <v>5673</v>
       </c>
       <c r="K32" t="n">
-        <v>1052</v>
+        <v>4156</v>
       </c>
     </row>
     <row r="33">
@@ -1162,16 +1147,16 @@
         </is>
       </c>
       <c r="G33" t="n">
-        <v>3463</v>
+        <v>2110</v>
       </c>
       <c r="H33" t="n">
-        <v>216</v>
-      </c>
-      <c r="I33" t="n">
-        <v>2855</v>
+        <v>2968</v>
       </c>
       <c r="J33" t="n">
-        <v>0</v>
+        <v>243</v>
+      </c>
+      <c r="K33" t="n">
+        <v>2757</v>
       </c>
     </row>
     <row r="34">
@@ -1183,17 +1168,17 @@
           <t>Taza de servicio x500</t>
         </is>
       </c>
-      <c r="G34" t="n">
-        <v>1378</v>
-      </c>
       <c r="H34" t="n">
-        <v>1018</v>
+        <v>1052</v>
+      </c>
+      <c r="I34" t="n">
+        <v>3463</v>
       </c>
       <c r="J34" t="n">
-        <v>4940</v>
+        <v>216</v>
       </c>
       <c r="K34" t="n">
-        <v>5422</v>
+        <v>2855</v>
       </c>
     </row>
     <row r="35">
@@ -1206,19 +1191,13 @@
         </is>
       </c>
       <c r="G35" t="n">
-        <v>3529</v>
-      </c>
-      <c r="H35" t="n">
-        <v>2966</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
-        <v>3139</v>
+        <v>1378</v>
       </c>
       <c r="J35" t="n">
-        <v>3498</v>
-      </c>
-      <c r="K35" t="n">
-        <v>1075</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="36">
@@ -1230,17 +1209,17 @@
           <t>Azúcar en stick x100</t>
         </is>
       </c>
-      <c r="G36" t="n">
-        <v>0</v>
+      <c r="H36" t="n">
+        <v>4940</v>
       </c>
       <c r="I36" t="n">
-        <v>4484</v>
+        <v>5422</v>
       </c>
       <c r="J36" t="n">
-        <v>3301</v>
+        <v>3529</v>
       </c>
       <c r="K36" t="n">
-        <v>1259</v>
+        <v>2966</v>
       </c>
     </row>
     <row r="37">
@@ -1253,16 +1232,16 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>185</v>
+        <v>3139</v>
       </c>
       <c r="H37" t="n">
-        <v>3972</v>
+        <v>3498</v>
       </c>
       <c r="I37" t="n">
-        <v>2628</v>
-      </c>
-      <c r="K37" t="n">
-        <v>782</v>
+        <v>1075</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -1274,17 +1253,17 @@
           <t>Azúcar en stick x100</t>
         </is>
       </c>
-      <c r="G38" t="n">
-        <v>4580</v>
+      <c r="H38" t="n">
+        <v>4484</v>
       </c>
       <c r="I38" t="n">
-        <v>4261</v>
+        <v>3301</v>
       </c>
       <c r="J38" t="n">
-        <v>2841</v>
+        <v>1259</v>
       </c>
       <c r="K38" t="n">
-        <v>2650</v>
+        <v>185</v>
       </c>
     </row>
     <row r="39">
@@ -1296,14 +1275,17 @@
           <t>Azúcar en stick x500</t>
         </is>
       </c>
+      <c r="G39" t="n">
+        <v>3972</v>
+      </c>
       <c r="H39" t="n">
-        <v>5193</v>
-      </c>
-      <c r="I39" t="n">
-        <v>3904</v>
+        <v>2628</v>
+      </c>
+      <c r="J39" t="n">
+        <v>782</v>
       </c>
       <c r="K39" t="n">
-        <v>4216</v>
+        <v>4580</v>
       </c>
     </row>
     <row r="40">
@@ -1315,20 +1297,14 @@
           <t>Taza de servicio x50</t>
         </is>
       </c>
-      <c r="G40" t="n">
-        <v>3319</v>
-      </c>
-      <c r="H40" t="n">
-        <v>2998</v>
-      </c>
       <c r="I40" t="n">
-        <v>1954</v>
+        <v>4261</v>
       </c>
       <c r="J40" t="n">
-        <v>2309</v>
+        <v>2841</v>
       </c>
       <c r="K40" t="n">
-        <v>1696</v>
+        <v>2650</v>
       </c>
     </row>
     <row r="41">
@@ -1340,20 +1316,14 @@
           <t>Azúcar en stick x50</t>
         </is>
       </c>
-      <c r="G41" t="n">
-        <v>3812</v>
-      </c>
       <c r="H41" t="n">
-        <v>4545</v>
+        <v>5193</v>
       </c>
       <c r="I41" t="n">
-        <v>5566</v>
-      </c>
-      <c r="J41" t="n">
-        <v>1589</v>
+        <v>3904</v>
       </c>
       <c r="K41" t="n">
-        <v>0</v>
+        <v>4216</v>
       </c>
     </row>
     <row r="42">
@@ -1365,20 +1335,17 @@
           <t>Taza de servicio x50</t>
         </is>
       </c>
-      <c r="G42" t="n">
-        <v>4021</v>
-      </c>
       <c r="H42" t="n">
-        <v>2953</v>
+        <v>3319</v>
       </c>
       <c r="I42" t="n">
-        <v>4336</v>
+        <v>2998</v>
       </c>
       <c r="J42" t="n">
-        <v>357</v>
+        <v>1954</v>
       </c>
       <c r="K42" t="n">
-        <v>739</v>
+        <v>2309</v>
       </c>
     </row>
     <row r="43">
@@ -1391,19 +1358,19 @@
         </is>
       </c>
       <c r="G43" t="n">
-        <v>4528</v>
+        <v>1696</v>
       </c>
       <c r="H43" t="n">
-        <v>1180</v>
+        <v>3812</v>
       </c>
       <c r="I43" t="n">
-        <v>875</v>
+        <v>4545</v>
       </c>
       <c r="J43" t="n">
-        <v>200</v>
+        <v>5566</v>
       </c>
       <c r="K43" t="n">
-        <v>5748</v>
+        <v>1589</v>
       </c>
     </row>
     <row r="44">
@@ -1415,17 +1382,17 @@
           <t>Paletina x500</t>
         </is>
       </c>
-      <c r="G44" t="n">
-        <v>4740</v>
+      <c r="H44" t="n">
+        <v>0</v>
       </c>
       <c r="I44" t="n">
-        <v>4465</v>
+        <v>4021</v>
       </c>
       <c r="J44" t="n">
-        <v>4281</v>
+        <v>2953</v>
       </c>
       <c r="K44" t="n">
-        <v>5471</v>
+        <v>4336</v>
       </c>
     </row>
     <row r="45">
@@ -1438,16 +1405,19 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>0</v>
+        <v>357</v>
       </c>
       <c r="H45" t="n">
-        <v>750</v>
+        <v>739</v>
+      </c>
+      <c r="I45" t="n">
+        <v>4528</v>
       </c>
       <c r="J45" t="n">
-        <v>4535</v>
+        <v>1180</v>
       </c>
       <c r="K45" t="n">
-        <v>390</v>
+        <v>875</v>
       </c>
     </row>
     <row r="46">
@@ -1459,17 +1429,14 @@
           <t>Paletina x500</t>
         </is>
       </c>
-      <c r="G46" t="n">
-        <v>5475</v>
-      </c>
       <c r="H46" t="n">
-        <v>1378</v>
+        <v>200</v>
       </c>
       <c r="I46" t="n">
-        <v>2469</v>
+        <v>5748</v>
       </c>
       <c r="J46" t="n">
-        <v>2976</v>
+        <v>4740</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Apertura debajo del canal: datos de prueba e importador
La base del mes anterior suma la hoja "Apertura anterior" en formato
largo (SKU, canal, entidad, kilos): distribuidores en Distribuidores y
vendedores en Directa, Córdoba y Rosario. Supuesto A10: cada territorio
con sus vendedores. Una entidad que no figura no aplica; 0 aplica con
cero. Formato de la apertura a confirmar (A3).

leer_apertura reporta entidades repetidas, repartos negativos y celdas
con error. El generador produce además celdas cuyas entidades tenían
todas 0 el mes anterior (entidad sin histórico, A4).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/sample/base_mes_anterior.xlsx
+++ b/data/sample/base_mes_anterior.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Distribución anterior" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Apertura anterior" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1442,4 +1443,3766 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D208"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Código SKU</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Canal</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Entidad</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Kilos</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>90020019</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Distribuidora Andina</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>90020019</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Distribuidora del Litoral</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>90020019</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Comercial Pampa</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>90020019</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Red Cuyo</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>90020019</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Norte Servicios</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>90020020</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Distribuidora Andina</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>897</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>90020020</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Distribuidora del Litoral</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>90020020</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Comercial Pampa</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>90020020</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Red Cuyo</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>90020020</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Norte Servicios</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>90020101</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Joaquín Ledesma</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>90020101</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Sofía Correa</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>90020101</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Nicolás Paz</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>90020101</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Tomás Quiroga</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>90020101</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Valentina Sosa</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>90020101</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Martín Acosta</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>90020101</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Camila Benítez</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>90020101</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Agustina Medina</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>90020101</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Federico Luna</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>90020102</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Joaquín Ledesma</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>90020102</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Sofía Correa</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>90020102</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Lucía Ferreyra</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>90020102</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Valentina Sosa</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>90020102</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Camila Benítez</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>90020102</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Distribuidora Andina</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>90020102</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Distribuidora del Litoral</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>881</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>90020102</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Comercial Pampa</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>90020102</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Norte Servicios</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>661</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>90020102</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Federico Luna</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>90020103</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Joaquín Ledesma</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>90020103</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Sofía Correa</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>90020103</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Nicolás Paz</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>90020103</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Lucía Ferreyra</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>90020103</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Valentina Sosa</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>90020103</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Martín Acosta</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>90020103</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Agustina Medina</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>90020103</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Federico Luna</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>90020104</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Joaquín Ledesma</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>90020104</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Sofía Correa</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>90020104</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Nicolás Paz</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>90020104</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Lucía Ferreyra</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>90020104</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Martín Acosta</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>90020104</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Agustina Medina</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>90020104</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Federico Luna</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>90020105</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Joaquín Ledesma</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>90020105</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Sofía Correa</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>90020105</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Nicolás Paz</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>90020105</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Lucía Ferreyra</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>90020105</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Tomás Quiroga</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>90020105</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Valentina Sosa</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>90020105</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Camila Benítez</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>90020105</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Agustina Medina</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>90020106</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Joaquín Ledesma</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>90020106</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Sofía Correa</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>90020106</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Nicolás Paz</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>90020106</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Tomás Quiroga</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>90020106</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Valentina Sosa</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>90020106</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Martín Acosta</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>90020106</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Camila Benítez</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>888</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>90020107</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Joaquín Ledesma</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>90020107</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Sofía Correa</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>883</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>90020107</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Nicolás Paz</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>90020107</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Lucía Ferreyra</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>90020107</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Tomás Quiroga</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>90020107</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Valentina Sosa</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>90020107</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Martín Acosta</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>90020107</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Camila Benítez</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>90020107</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Agustina Medina</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>90020107</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Federico Luna</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>90020108</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Joaquín Ledesma</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>90020108</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Sofía Correa</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>90020108</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Nicolás Paz</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>90020108</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Distribuidora Andina</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>886</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>90020108</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Distribuidora del Litoral</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>90020108</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Comercial Pampa</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>90020108</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Red Cuyo</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>90020108</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Norte Servicios</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>90020108</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Federico Luna</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>887</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>90020109</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Joaquín Ledesma</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>90020109</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Sofía Correa</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>90020109</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Nicolás Paz</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>90020110</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Sofía Correa</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>90020110</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Nicolás Paz</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>90020110</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Lucía Ferreyra</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>90020110</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Tomás Quiroga</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>90020110</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Valentina Sosa</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>90020110</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Camila Benítez</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>90020110</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Distribuidora del Litoral</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>90020110</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Comercial Pampa</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>90020110</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Red Cuyo</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>90020110</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Norte Servicios</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>779</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>90020111</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Joaquín Ledesma</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>90020111</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Sofía Correa</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>90020111</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Nicolás Paz</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>90020111</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Lucía Ferreyra</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>90020111</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Valentina Sosa</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>90020111</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Camila Benítez</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>90020111</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Agustina Medina</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>90020112</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Tomás Quiroga</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>90020112</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Valentina Sosa</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>90020112</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Martín Acosta</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>90020112</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Distribuidora Andina</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>899</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>90020112</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Distribuidora del Litoral</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>90020112</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Comercial Pampa</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>90020112</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Red Cuyo</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>90020112</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Norte Servicios</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>90020112</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Agustina Medina</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>90020112</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Federico Luna</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>90020113</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Sofía Correa</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>90020113</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Nicolás Paz</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>90020113</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Lucía Ferreyra</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>90020113</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Tomás Quiroga</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>90020113</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Valentina Sosa</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>90020113</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Martín Acosta</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>90020113</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Camila Benítez</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>90020113</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Agustina Medina</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>90020113</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Federico Luna</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>90020114</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Joaquín Ledesma</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>90020114</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Sofía Correa</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>90020114</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Nicolás Paz</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>90020114</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Federico Luna</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>90020115</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Joaquín Ledesma</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>90020115</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Nicolás Paz</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>90020115</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Lucía Ferreyra</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>90020115</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Tomás Quiroga</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>90020115</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Valentina Sosa</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>90020115</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Camila Benítez</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>90020115</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Agustina Medina</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>90020115</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Federico Luna</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>90020116</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Joaquín Ledesma</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>90020116</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Sofía Correa</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>90020116</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Nicolás Paz</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>90020116</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Lucía Ferreyra</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>90020116</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Valentina Sosa</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>90020116</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Martín Acosta</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>90020116</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Camila Benítez</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>90020116</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Distribuidora Andina</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>90020116</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Distribuidora del Litoral</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>90020116</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Comercial Pampa</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>90020116</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Red Cuyo</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>843</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>90020116</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Norte Servicios</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>90020117</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Nicolás Paz</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>90020117</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Lucía Ferreyra</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>90020117</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Tomás Quiroga</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>829</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>90020117</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Valentina Sosa</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>90020117</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Martín Acosta</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>90020117</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Agustina Medina</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>90020118</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Lucía Ferreyra</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>90020118</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Tomás Quiroga</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>90020118</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Camila Benítez</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>90020118</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Distribuidora Andina</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>90020118</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Distribuidora del Litoral</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>887</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>90020118</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Comercial Pampa</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>90020118</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Norte Servicios</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>90020118</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Agustina Medina</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>90020118</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Federico Luna</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>90020119</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Joaquín Ledesma</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>90020119</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Sofía Correa</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>90020119</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Nicolás Paz</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>90020119</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Agustina Medina</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>90020120</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Nicolás Paz</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>90020120</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Lucía Ferreyra</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>90020120</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Tomás Quiroga</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>90020120</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Valentina Sosa</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>90020120</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Martín Acosta</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>90020121</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Joaquín Ledesma</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="n">
+        <v>90020121</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Sofía Correa</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>90020121</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Nicolás Paz</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>90020121</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Lucía Ferreyra</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>90020121</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Tomás Quiroga</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>90020121</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Valentina Sosa</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>90020121</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Camila Benítez</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>90020121</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Agustina Medina</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>90020122</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Joaquín Ledesma</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>90020122</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Sofía Correa</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>90020122</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Nicolás Paz</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>90020122</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Lucía Ferreyra</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>90020122</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Valentina Sosa</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>829</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>90020122</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Camila Benítez</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>90020122</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Comercial Pampa</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>90020122</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Red Cuyo</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>90020122</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Norte Servicios</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>90020122</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Federico Luna</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>90020123</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Sofía Correa</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>90020123</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Nicolás Paz</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>90020123</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Agustina Medina</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>90020123</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Federico Luna</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>889</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>90020124</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Joaquín Ledesma</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>90020124</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Sofía Correa</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>90020124</v>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Tomás Quiroga</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>90020124</v>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Valentina Sosa</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>90020124</v>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Martín Acosta</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>90020124</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Distribuidora Andina</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>90020124</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Distribuidora del Litoral</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>90020124</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Comercial Pampa</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>90020124</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Red Cuyo</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>90020124</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Distribuidores</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Norte Servicios</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>90020124</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Agustina Medina</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>90020124</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Federico Luna</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>90020125</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Joaquín Ledesma</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>90020125</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Sofía Correa</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>90020125</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Lucía Ferreyra</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="n">
+        <v>90020125</v>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Tomás Quiroga</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="n">
+        <v>90020125</v>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Martín Acosta</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="n">
+        <v>90020125</v>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Directa (BA)</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Camila Benítez</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="n">
+        <v>90020125</v>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Agustina Medina</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
+        <v>90020125</v>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Rosario</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Federico Luna</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>671</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>